<commit_message>
Grade 9 Set A: replace gerund question with journey vocabulary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012At1DdBHCbmKTSWhAZPRk5
</commit_message>
<xml_diff>
--- a/sets/grade9-theme1-set1/questions.xlsx
+++ b/sets/grade9-theme1-set1/questions.xlsx
@@ -1410,28 +1410,28 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Nora is a vlogger. She goes ______ in Santiago and takes photos.</t>
+          <t>Nora's ______ lasts two months. She visits many different countries.</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>visit</t>
+          <t>palace</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>to sightseeing</t>
+          <t>ruin</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>sightsee</t>
+          <t>tower</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>sightseeing</t>
+          <t>journey</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>go + -ing: go swimming, go hiking…</t>
+          <t>a long trip</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr"/>

</xml_diff>